<commit_message>
Document what the OneDrive sync can and cannot automate
Leer el .xlsx desde OneDrive funciona: el conector devuelve el contenido como
filas tabuladas por hoja, suficiente para reconstruir las tablas y reescribir
los YAML. Escribirlo de vuelta no: exige pasar el binario completo en base64
dentro de la conversación y el entorno deja fuera de contexto las salidas de
ese tamaño.

El README y la hoja «Léeme» describían el paso 4 como una subida automática.
Corregido en ambos sitios para que el ciclo documentado sea el que de verdad
se puede ejecutar.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gtsxhnze1SF7LaG9UGLdD2
</commit_message>
<xml_diff>
--- a/growth-os/dist/Founderz_Growth_OS.xlsx
+++ b/growth-os/dist/Founderz_Growth_OS.xlsx
@@ -1146,14 +1146,14 @@
     <row r="8" ht="30" customHeight="1">
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>3. Le dices al agente «sincroniza el Growth OS». El agente lee el Excel, actualiza los YAML del repo y hace commit: ahí queda el histórico.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
+          <t>3. Le dices al agente «sincroniza el Growth OS». El agente lee el Excel desde OneDrive, actualiza los YAML del repo y hace commit: ahí queda el histórico.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>4. Cuando hay cambios estructurales (nuevos departamentos, columnas, métricas o reglas de cálculo), el agente regenera el Excel y lo vuelve a subir.</t>
+          <t>4. Cuando hay cambios estructurales (nuevos departamentos, columnas, métricas o reglas de cálculo), el agente regenera el fichero y te lo entrega para que lo dejes en la carpeta. Sustituye el anterior y sigues trabajando.</t>
         </is>
       </c>
     </row>

</xml_diff>